<commit_message>
Correction Montant_Exclu_Rejet BSA : NON_REMB - TPG
Pour BSA, le NON_REMB du PDF inclut le TPG (ticket modérateur).
Le vrai montant exclu/rejet = NON_REMB - TPG.
Cohérence vérifiée : FR.REELS = REMB + (NON_REMB - TPG) sur toutes les lignes.

- BSA_paiement_to_excel.py : Montant_Exclu_Rejet = max(0, num(nonremb) - num(tpg))
- Fichier Excel BSA 2025 régénéré avec les valeurs corrigées
- Documentation mise à jour dans les docstrings

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PAIEMENT CLIENT/BSA/2025/16-09-25 BSA 2025 05-06-25 à 29-07-25 MONTANT 777 650Ar.xlsx
+++ b/PAIEMENT CLIENT/BSA/2025/16-09-25 BSA 2025 05-06-25 à 29-07-25 MONTANT 777 650Ar.xlsx
@@ -555,7 +555,7 @@
         <v>80000</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="M2" s="1" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
         <v>20000</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="M6" s="1" t="inlineStr">
         <is>
@@ -1778,7 +1778,7 @@
         <v>20000</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="M23" s="1" t="inlineStr">
         <is>
@@ -2132,7 +2132,7 @@
         <v>20000</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="M29" s="1" t="inlineStr">
         <is>
@@ -2777,7 +2777,7 @@
         <v>20000</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="M40" s="1" t="inlineStr">
         <is>
@@ -3013,7 +3013,7 @@
         <v>20000</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="M44" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(BSA): corriger mapping Ticket_Moderateur et ajouter vérification de cohérence
- Ticket_Moderateur = Tx (%) au lieu de TPG (taux de prise en charge)
- Montant_Reclame_Brut = FR.REELS
- Montant_Paye_Regle = REMB
- Montant_Exclu_Rejet = NON_REMB - TPG (montant exclu réel)
- Ajout d'un contrôle de cohérence automatique par ligne :
  FR.REELS = REMB + (NON_REMB - TPG)
- Documentation mise à jour (VERIFICATION_BSA.md, RESUME_MODIFICATIONS_BSA.txt)

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PAIEMENT CLIENT/BSA/2025/16-09-25 BSA 2025 05-06-25 à 29-07-25 MONTANT 777 650Ar.xlsx
+++ b/PAIEMENT CLIENT/BSA/2025/16-09-25 BSA 2025 05-06-25 à 29-07-25 MONTANT 777 650Ar.xlsx
@@ -549,7 +549,7 @@
         <v>80000</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>20000</v>
+        <v>100</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>80000</v>
@@ -608,7 +608,7 @@
         <v>10000</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>10000</v>
@@ -663,7 +663,7 @@
         <v>5000</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>5000</v>
@@ -718,7 +718,7 @@
         <v>156900</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>156900</v>
@@ -777,7 +777,7 @@
         <v>20000</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>5000</v>
+        <v>95</v>
       </c>
       <c r="K6" s="2" t="n">
         <v>20000</v>
@@ -836,7 +836,7 @@
         <v>12000</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>12000</v>
@@ -895,7 +895,7 @@
         <v>1500</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>1500</v>
@@ -954,7 +954,7 @@
         <v>10800</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>10800</v>
@@ -1013,7 +1013,7 @@
         <v>20000</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>15000</v>
@@ -1072,7 +1072,7 @@
         <v>40500</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>40500</v>
@@ -1131,7 +1131,7 @@
         <v>10000</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>10000</v>
@@ -1190,7 +1190,7 @@
         <v>5500</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>5500</v>
@@ -1249,7 +1249,7 @@
         <v>20000</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="K14" s="2" t="n">
         <v>15000</v>
@@ -1308,7 +1308,7 @@
         <v>12000</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K15" s="2" t="n">
         <v>12000</v>
@@ -1367,7 +1367,7 @@
         <v>8000</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>8000</v>
@@ -1426,7 +1426,7 @@
         <v>12000</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K17" s="2" t="n">
         <v>12000</v>
@@ -1481,7 +1481,7 @@
         <v>12000</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K18" s="2" t="n">
         <v>12000</v>
@@ -1536,7 +1536,7 @@
         <v>15000</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="K19" s="2" t="n">
         <v>14250</v>
@@ -1595,7 +1595,7 @@
         <v>6000</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>6000</v>
@@ -1654,7 +1654,7 @@
         <v>28600</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K21" s="2" t="n">
         <v>28600</v>
@@ -1713,7 +1713,7 @@
         <v>15000</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K22" s="2" t="n">
         <v>15000</v>
@@ -1772,7 +1772,7 @@
         <v>20000</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>5000</v>
+        <v>95</v>
       </c>
       <c r="K23" s="2" t="n">
         <v>20000</v>
@@ -1831,7 +1831,7 @@
         <v>6000</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K24" s="2" t="n">
         <v>6000</v>
@@ -1890,7 +1890,7 @@
         <v>24000</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K25" s="2" t="n">
         <v>24000</v>
@@ -1949,7 +1949,7 @@
         <v>25000</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K26" s="2" t="n">
         <v>25000</v>
@@ -2008,7 +2008,7 @@
         <v>1500</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>1500</v>
@@ -2067,7 +2067,7 @@
         <v>26000</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>26000</v>
@@ -2126,7 +2126,7 @@
         <v>20000</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>5000</v>
+        <v>95</v>
       </c>
       <c r="K29" s="2" t="n">
         <v>20000</v>
@@ -2185,7 +2185,7 @@
         <v>1500</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K30" s="2" t="n">
         <v>1500</v>
@@ -2244,7 +2244,7 @@
         <v>1500</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>1500</v>
@@ -2303,7 +2303,7 @@
         <v>1500</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>1500</v>
@@ -2362,7 +2362,7 @@
         <v>16000</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K33" s="2" t="n">
         <v>16000</v>
@@ -2421,7 +2421,7 @@
         <v>9600</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K34" s="2" t="n">
         <v>9600</v>
@@ -2771,7 +2771,7 @@
         <v>20000</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>5000</v>
+        <v>95</v>
       </c>
       <c r="K40" s="2" t="n">
         <v>20000</v>
@@ -2830,7 +2830,7 @@
         <v>6000</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K41" s="2" t="n">
         <v>6000</v>
@@ -2889,7 +2889,7 @@
         <v>12500</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K42" s="2" t="n">
         <v>12500</v>
@@ -2948,7 +2948,7 @@
         <v>10400</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K43" s="2" t="n">
         <v>10400</v>
@@ -3007,7 +3007,7 @@
         <v>20000</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>5000</v>
+        <v>95</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>20000</v>
@@ -3066,7 +3066,7 @@
         <v>8500</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>8500</v>
@@ -3125,7 +3125,7 @@
         <v>9600</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>9600</v>
@@ -3184,7 +3184,7 @@
         <v>6000</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>6000</v>
@@ -3243,7 +3243,7 @@
         <v>1000</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K48" s="2" t="n">
         <v>1000</v>
@@ -3298,7 +3298,7 @@
         <v>3000</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K49" s="2" t="n">
         <v>3000</v>
@@ -3357,7 +3357,7 @@
         <v>15000</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>15000</v>
@@ -3412,7 +3412,7 @@
         <v>3000</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>3000</v>
@@ -3471,7 +3471,7 @@
         <v>20000</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>20000</v>

</xml_diff>